<commit_message>
Stock Check for Target price
</commit_message>
<xml_diff>
--- a/nseshare/stocks.xlsx
+++ b/nseshare/stocks.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+  <workbookPr filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -19,32 +19,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>DCBBank</t>
-  </si>
-  <si>
-    <t>HAPPMINDS</t>
-  </si>
-  <si>
-    <t>HCLTECH</t>
-  </si>
-  <si>
-    <t>INFY</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>ITC</t>
   </si>
   <si>
-    <t>JKPAPER</t>
-  </si>
-  <si>
-    <t>KANANIIND</t>
-  </si>
-  <si>
-    <t>KOHINOOR</t>
-  </si>
-  <si>
     <t>TargetPrice</t>
   </si>
   <si>
@@ -52,12 +31,81 @@
   </si>
   <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>HEROMOTOCO</t>
+  </si>
+  <si>
+    <t>SHRIRAMPPS</t>
+  </si>
+  <si>
+    <t>KTKBANK</t>
+  </si>
+  <si>
+    <t>PRESTIGE</t>
+  </si>
+  <si>
+    <t>TATACHEM</t>
+  </si>
+  <si>
+    <t>SPANDANA</t>
+  </si>
+  <si>
+    <t>FEDERALBNK</t>
+  </si>
+  <si>
+    <t>BORORENEW</t>
+  </si>
+  <si>
+    <t>SEKURITIND</t>
+  </si>
+  <si>
+    <t>IDFCFIRSTB</t>
+  </si>
+  <si>
+    <t>MUTHOOTFIN</t>
+  </si>
+  <si>
+    <t>TATAGOLD</t>
+  </si>
+  <si>
+    <t>ZYDUSLIFE</t>
+  </si>
+  <si>
+    <t>MON100</t>
+  </si>
+  <si>
+    <t>THANGAMAYL</t>
+  </si>
+  <si>
+    <t>TITAN</t>
+  </si>
+  <si>
+    <t>SOUTHBANK</t>
+  </si>
+  <si>
+    <t>RTNPOWER</t>
+  </si>
+  <si>
+    <t>TATATECH</t>
+  </si>
+  <si>
+    <t>HERITGFOOD</t>
+  </si>
+  <si>
+    <t>GODREJPROP</t>
+  </si>
+  <si>
+    <t>AXISBANK</t>
+  </si>
+  <si>
+    <t>MANAPPURAM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -87,9 +135,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -370,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -378,13 +427,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -392,10 +441,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C2" s="1">
-        <v>100</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -403,10 +452,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1">
-        <v>780</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -414,10 +463,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1">
-        <v>1100</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -425,10 +474,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C5" s="1">
-        <v>1700</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -436,10 +485,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C6" s="1">
-        <v>500</v>
+        <v>380.75</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -447,10 +496,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C7" s="1">
-        <v>380</v>
+        <v>750</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -458,10 +507,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C8" s="1">
-        <v>3</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -469,13 +518,475 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C9" s="1">
-        <v>3835</v>
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="2">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="2">
+        <v>65.400000000000006</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="2">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="2">
+        <v>2986</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="2">
+        <v>22.99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="2">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="2">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="2">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="2">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="2">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>